<commit_message>
docs(bloc3): ancrer le pilotage dans Linear et détailler les estimations
</commit_message>
<xml_diff>
--- a/outputs/bloc03-01a09eba/pilotage-spity.xlsx
+++ b/outputs/bloc03-01a09eba/pilotage-spity.xlsx
@@ -2,9 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilotage" sheetId="1" r:id="R4304f672b45d4a0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planning" sheetId="2" r:id="Rf4898173b7894517"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risques" sheetId="3" r:id="Rd90249566a584024"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilotage" sheetId="1" r:id="Rf5ef7024ad4641f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planning" sheetId="2" r:id="Rae6a336d5a514871"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risques" sheetId="3" r:id="R77f82d07d8ca47f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimations" sheetId="4" r:id="Racdf1b04fcce417b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Linear" sheetId="5" r:id="Rabe8b91f510f4c43"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,11 +17,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="0.0%"/>
     <x:numFmt numFmtId="201" formatCode="#,##0 &quot;€&quot;;(#,##0) &quot;€&quot;;&quot;-&quot;"/>
     <x:numFmt numFmtId="202" formatCode="0%"/>
     <x:numFmt numFmtId="203" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
+    <x:numFmt numFmtId="204" formatCode="#,##0 &quot;€&quot;"/>
   </x:numFmts>
   <x:fonts count="7">
     <x:font>
@@ -89,7 +92,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="24">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -146,6 +149,9 @@
     <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="204" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
@@ -155,6 +161,9 @@
     <x:xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
@@ -162,7 +171,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="5">
+  <x:dxfs count="6">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -171,6 +180,17 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFDE5CD"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA32121"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE2E2"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -718,7 +738,7 @@
       </x:c>
       <x:c r="D18" s="2"/>
       <x:c r="E18" s="2" t="str">
-        <x:v>Archive Linear du 09/09/2026 : 12 Done / 24 actifs.</x:v>
+        <x:v>Linear lu le 14/09/2026 : 12 Done / 24 non annulés.</x:v>
       </x:c>
       <x:c r="F18" s="2"/>
       <x:c r="G18" s="2"/>
@@ -738,7 +758,7 @@
       </x:c>
       <x:c r="D19" s="2"/>
       <x:c r="E19" s="2" t="str">
-        <x:v>Cette archive est distincte des 10 tâches simulées.</x:v>
+        <x:v>Statuts observés dans la feuille Linear ; cas distinct.</x:v>
       </x:c>
       <x:c r="F19" s="2"/>
       <x:c r="G19" s="2"/>
@@ -1109,6 +1129,188 @@
       <x:c r="K36" s="2"/>
       <x:c r="L36" s="2"/>
     </x:row>
+    <x:row r="37" ht="25" customHeight="1">
+      <x:c r="B37" s="2" t="str">
+        <x:v>Sensibilité : une hypothèse ajoutée à la fois à J10</x:v>
+      </x:c>
+      <x:c r="C37" s="2"/>
+      <x:c r="D37" s="2"/>
+      <x:c r="E37" s="2"/>
+      <x:c r="F37" s="2"/>
+      <x:c r="G37" s="2"/>
+      <x:c r="H37" s="2"/>
+    </x:row>
+    <x:row r="38" ht="25" customHeight="1">
+      <x:c r="B38" s="2"/>
+      <x:c r="C38" s="2"/>
+      <x:c r="D38" s="2"/>
+      <x:c r="E38" s="2"/>
+      <x:c r="F38" s="2"/>
+      <x:c r="G38" s="2"/>
+      <x:c r="H38" s="2"/>
+    </x:row>
+    <x:row r="39" ht="36" customHeight="1">
+      <x:c r="B39" s="7" t="str">
+        <x:v>Hypothèse</x:v>
+      </x:c>
+      <x:c r="C39" s="7" t="str">
+        <x:v>CP +h</x:v>
+      </x:c>
+      <x:c r="D39" s="7" t="str">
+        <x:v>DEV +h</x:v>
+      </x:c>
+      <x:c r="E39" s="7" t="str">
+        <x:v>QA +h</x:v>
+      </x:c>
+      <x:c r="F39" s="7" t="str">
+        <x:v>Prévision EUR</x:v>
+      </x:c>
+      <x:c r="G39" s="7" t="str">
+        <x:v>Marge EUR</x:v>
+      </x:c>
+      <x:c r="H39" s="7" t="str">
+        <x:v>Capacité dépassée</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="25" customHeight="1">
+      <x:c r="B40" s="2" t="str">
+        <x:v>Prévision J10</x:v>
+      </x:c>
+      <x:c r="C40" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D40" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E40" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F40" s="20" t="n">
+        <x:f>$C$16+C40*$D$23+D40*$D$24+E40*$D$25</x:f>
+        <x:v>4465</x:v>
+      </x:c>
+      <x:c r="G40" s="20" t="n">
+        <x:f>$C$18-F40</x:f>
+        <x:v>232</x:v>
+      </x:c>
+      <x:c r="H40" s="2" t="str">
+        <x:f>IF($H$23+C40&gt;$C$23,"CP",IF($H$24+D40&gt;$C$24,"DEV",IF($H$25+E40&gt;$C$25,"QA","Aucune")))</x:f>
+        <x:v>Aucune</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="25" customHeight="1">
+      <x:c r="B41" s="2" t="str">
+        <x:v>Recette +6 h</x:v>
+      </x:c>
+      <x:c r="C41" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D41" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E41" s="18" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F41" s="20" t="n">
+        <x:f>$C$16+C41*$D$23+D41*$D$24+E41*$D$25</x:f>
+        <x:v>4645</x:v>
+      </x:c>
+      <x:c r="G41" s="20" t="n">
+        <x:f>$C$18-F41</x:f>
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="H41" s="2" t="str">
+        <x:f>IF($H$23+C41&gt;$C$23,"CP",IF($H$24+D41&gt;$C$24,"DEV",IF($H$25+E41&gt;$C$25,"QA","Aucune")))</x:f>
+        <x:v>Aucune</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="25" customHeight="1">
+      <x:c r="B42" s="2" t="str">
+        <x:v>DEV +8 h</x:v>
+      </x:c>
+      <x:c r="C42" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D42" s="18" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E42" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F42" s="20" t="n">
+        <x:f>$C$16+C42*$D$23+D42*$D$24+E42*$D$25</x:f>
+        <x:v>4745</x:v>
+      </x:c>
+      <x:c r="G42" s="20" t="n">
+        <x:f>$C$18-F42</x:f>
+        <x:v>-48</x:v>
+      </x:c>
+      <x:c r="H42" s="2" t="str">
+        <x:f>IF($H$23+C42&gt;$C$23,"CP",IF($H$24+D42&gt;$C$24,"DEV",IF($H$25+E42&gt;$C$25,"QA","Aucune")))</x:f>
+        <x:v>Aucune</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="25" customHeight="1">
+      <x:c r="B43" s="2" t="str">
+        <x:v>CP +2 h</x:v>
+      </x:c>
+      <x:c r="C43" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D43" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E43" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F43" s="20" t="n">
+        <x:f>$C$16+C43*$D$23+D43*$D$24+E43*$D$25</x:f>
+        <x:v>4555</x:v>
+      </x:c>
+      <x:c r="G43" s="20" t="n">
+        <x:f>$C$18-F43</x:f>
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="H43" s="2" t="str">
+        <x:f>IF($H$23+C43&gt;$C$23,"CP",IF($H$24+D43&gt;$C$24,"DEV",IF($H$25+E43&gt;$C$25,"QA","Aucune")))</x:f>
+        <x:v>CP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="25" customHeight="1">
+      <x:c r="B44" s="2" t="str">
+        <x:v>Topo +16 h</x:v>
+      </x:c>
+      <x:c r="C44" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D44" s="18" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E44" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F44" s="20" t="n">
+        <x:f>$C$16+C44*$D$23+D44*$D$24+E44*$D$25</x:f>
+        <x:v>5005</x:v>
+      </x:c>
+      <x:c r="G44" s="20" t="n">
+        <x:f>$C$18-F44</x:f>
+        <x:v>-308</x:v>
+      </x:c>
+      <x:c r="H44" s="2" t="str">
+        <x:f>IF($H$23+C44&gt;$C$23,"CP",IF($H$24+D44&gt;$C$24,"DEV",IF($H$25+E44&gt;$C$25,"QA","Aucune")))</x:f>
+        <x:v>DEV</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="25" customHeight="1">
+      <x:c r="B45" s="2"/>
+      <x:c r="C45" s="2"/>
+      <x:c r="D45" s="2"/>
+      <x:c r="E45" s="2"/>
+      <x:c r="F45" s="2"/>
+      <x:c r="G45" s="2"/>
+      <x:c r="H45" s="2"/>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="L23:L25">
     <x:cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
@@ -1117,6 +1319,11 @@
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="C19:C19">
     <x:cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
+      <x:formula>0</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G40:G44">
+    <x:cfRule type="cellIs" dxfId="2" priority="3" operator="lessThan">
       <x:formula>0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -1300,25 +1507,28 @@
       <x:c r="C9" s="2" t="str">
         <x:v>CP</x:v>
       </x:c>
-      <x:c r="D9" s="22" t="n">
+      <x:c r="D9" s="23" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E9" s="22" t="n">
+      <x:c r="E9" s="23" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F9" s="22" t="n">
+      <x:c r="F9" s="23" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="G9" s="18" t="str">
         <x:v>Terminé</x:v>
       </x:c>
-      <x:c r="H9" s="18" t="n">
+      <x:c r="H9" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$E$9:$E$38)=30,SUMIFS('Estimations'!$E$9:$E$38,'Estimations'!$B$9:$B$38,A9),NA())</x:f>
         <x:v>6</x:v>
       </x:c>
-      <x:c r="I9" s="18" t="n">
+      <x:c r="I9" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$F$9:$F$38)=30,SUMIFS('Estimations'!$F$9:$F$38,'Estimations'!$B$9:$B$38,A9),NA())</x:f>
         <x:v>6</x:v>
       </x:c>
-      <x:c r="J9" s="18" t="n">
+      <x:c r="J9" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$G$9:$G$38)=30,SUMIFS('Estimations'!$G$9:$G$38,'Estimations'!$B$9:$B$38,A9),NA())</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K9" s="2" t="n">
@@ -1329,10 +1539,10 @@
         <x:f>K9-H9</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M9" s="20" t="str">
+      <x:c r="M9" s="21" t="str">
         <x:v>Aucun</x:v>
       </x:c>
-      <x:c r="N9" s="20" t="n">
+      <x:c r="N9" s="21" t="n">
         <x:f>F9-E9</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1347,25 +1557,28 @@
       <x:c r="C10" s="2" t="str">
         <x:v>QA</x:v>
       </x:c>
-      <x:c r="D10" s="22" t="n">
+      <x:c r="D10" s="23" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E10" s="22" t="n">
+      <x:c r="E10" s="23" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="F10" s="22" t="n">
+      <x:c r="F10" s="23" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="G10" s="18" t="str">
         <x:v>Terminé</x:v>
       </x:c>
-      <x:c r="H10" s="18" t="n">
+      <x:c r="H10" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$E$9:$E$38)=30,SUMIFS('Estimations'!$E$9:$E$38,'Estimations'!$B$9:$B$38,A10),NA())</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="I10" s="18" t="n">
+      <x:c r="I10" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$F$9:$F$38)=30,SUMIFS('Estimations'!$F$9:$F$38,'Estimations'!$B$9:$B$38,A10),NA())</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="J10" s="18" t="n">
+      <x:c r="J10" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$G$9:$G$38)=30,SUMIFS('Estimations'!$G$9:$G$38,'Estimations'!$B$9:$B$38,A10),NA())</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K10" s="2" t="n">
@@ -1376,10 +1589,10 @@
         <x:f>K10-H10</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M10" s="20" t="str">
+      <x:c r="M10" s="21" t="str">
         <x:v>Aucun</x:v>
       </x:c>
-      <x:c r="N10" s="20" t="n">
+      <x:c r="N10" s="21" t="n">
         <x:f>F10-E10</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1394,25 +1607,28 @@
       <x:c r="C11" s="2" t="str">
         <x:v>CP</x:v>
       </x:c>
-      <x:c r="D11" s="22" t="n">
+      <x:c r="D11" s="23" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="E11" s="22" t="n">
+      <x:c r="E11" s="23" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="F11" s="22" t="n">
+      <x:c r="F11" s="23" t="n">
         <x:v>4</x:v>
       </x:c>
       <x:c r="G11" s="18" t="str">
         <x:v>Terminé</x:v>
       </x:c>
-      <x:c r="H11" s="18" t="n">
+      <x:c r="H11" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$E$9:$E$38)=30,SUMIFS('Estimations'!$E$9:$E$38,'Estimations'!$B$9:$B$38,A11),NA())</x:f>
         <x:v>6</x:v>
       </x:c>
-      <x:c r="I11" s="18" t="n">
+      <x:c r="I11" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$F$9:$F$38)=30,SUMIFS('Estimations'!$F$9:$F$38,'Estimations'!$B$9:$B$38,A11),NA())</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="J11" s="18" t="n">
+      <x:c r="J11" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$G$9:$G$38)=30,SUMIFS('Estimations'!$G$9:$G$38,'Estimations'!$B$9:$B$38,A11),NA())</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K11" s="2" t="n">
@@ -1423,10 +1639,10 @@
         <x:f>K11-H11</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M11" s="20" t="str">
+      <x:c r="M11" s="21" t="str">
         <x:v>Aucun</x:v>
       </x:c>
-      <x:c r="N11" s="20" t="n">
+      <x:c r="N11" s="21" t="n">
         <x:f>F11-E11</x:f>
         <x:v>1</x:v>
       </x:c>
@@ -1441,25 +1657,28 @@
       <x:c r="C12" s="2" t="str">
         <x:v>DEV</x:v>
       </x:c>
-      <x:c r="D12" s="22" t="n">
+      <x:c r="D12" s="23" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E12" s="22" t="n">
+      <x:c r="E12" s="23" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F12" s="22" t="n">
+      <x:c r="F12" s="23" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="G12" s="18" t="str">
         <x:v>Terminé</x:v>
       </x:c>
-      <x:c r="H12" s="18" t="n">
+      <x:c r="H12" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$E$9:$E$38)=30,SUMIFS('Estimations'!$E$9:$E$38,'Estimations'!$B$9:$B$38,A12),NA())</x:f>
         <x:v>18</x:v>
       </x:c>
-      <x:c r="I12" s="18" t="n">
+      <x:c r="I12" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$F$9:$F$38)=30,SUMIFS('Estimations'!$F$9:$F$38,'Estimations'!$B$9:$B$38,A12),NA())</x:f>
         <x:v>20</x:v>
       </x:c>
-      <x:c r="J12" s="18" t="n">
+      <x:c r="J12" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$G$9:$G$38)=30,SUMIFS('Estimations'!$G$9:$G$38,'Estimations'!$B$9:$B$38,A12),NA())</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K12" s="2" t="n">
@@ -1470,10 +1689,10 @@
         <x:f>K12-H12</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="M12" s="20" t="str">
+      <x:c r="M12" s="21" t="str">
         <x:v>T01</x:v>
       </x:c>
-      <x:c r="N12" s="20" t="n">
+      <x:c r="N12" s="21" t="n">
         <x:f>F12-E12</x:f>
         <x:v>1</x:v>
       </x:c>
@@ -1488,25 +1707,28 @@
       <x:c r="C13" s="2" t="str">
         <x:v>DEV</x:v>
       </x:c>
-      <x:c r="D13" s="22" t="n">
+      <x:c r="D13" s="23" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="E13" s="22" t="n">
+      <x:c r="E13" s="23" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="F13" s="22" t="n">
+      <x:c r="F13" s="23" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="G13" s="18" t="str">
         <x:v>Terminé</x:v>
       </x:c>
-      <x:c r="H13" s="18" t="n">
+      <x:c r="H13" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$E$9:$E$38)=30,SUMIFS('Estimations'!$E$9:$E$38,'Estimations'!$B$9:$B$38,A13),NA())</x:f>
         <x:v>16</x:v>
       </x:c>
-      <x:c r="I13" s="18" t="n">
+      <x:c r="I13" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$F$9:$F$38)=30,SUMIFS('Estimations'!$F$9:$F$38,'Estimations'!$B$9:$B$38,A13),NA())</x:f>
         <x:v>16</x:v>
       </x:c>
-      <x:c r="J13" s="18" t="n">
+      <x:c r="J13" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$G$9:$G$38)=30,SUMIFS('Estimations'!$G$9:$G$38,'Estimations'!$B$9:$B$38,A13),NA())</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K13" s="2" t="n">
@@ -1517,10 +1739,10 @@
         <x:f>K13-H13</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M13" s="20" t="str">
+      <x:c r="M13" s="21" t="str">
         <x:v>T04</x:v>
       </x:c>
-      <x:c r="N13" s="20" t="n">
+      <x:c r="N13" s="21" t="n">
         <x:f>F13-E13</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1535,25 +1757,28 @@
       <x:c r="C14" s="2" t="str">
         <x:v>DEV</x:v>
       </x:c>
-      <x:c r="D14" s="22" t="n">
+      <x:c r="D14" s="23" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E14" s="22" t="n">
+      <x:c r="E14" s="23" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F14" s="22" t="n">
+      <x:c r="F14" s="23" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="G14" s="18" t="str">
         <x:v>En cours</x:v>
       </x:c>
-      <x:c r="H14" s="18" t="n">
+      <x:c r="H14" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$E$9:$E$38)=30,SUMIFS('Estimations'!$E$9:$E$38,'Estimations'!$B$9:$B$38,A14),NA())</x:f>
         <x:v>18</x:v>
       </x:c>
-      <x:c r="I14" s="18" t="n">
+      <x:c r="I14" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$F$9:$F$38)=30,SUMIFS('Estimations'!$F$9:$F$38,'Estimations'!$B$9:$B$38,A14),NA())</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="J14" s="18" t="n">
+      <x:c r="J14" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$G$9:$G$38)=30,SUMIFS('Estimations'!$G$9:$G$38,'Estimations'!$B$9:$B$38,A14),NA())</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="K14" s="2" t="n">
@@ -1564,10 +1789,10 @@
         <x:f>K14-H14</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="M14" s="20" t="str">
+      <x:c r="M14" s="21" t="str">
         <x:v>T05</x:v>
       </x:c>
-      <x:c r="N14" s="20" t="n">
+      <x:c r="N14" s="21" t="n">
         <x:f>F14-E14</x:f>
         <x:v>1</x:v>
       </x:c>
@@ -1582,25 +1807,28 @@
       <x:c r="C15" s="2" t="str">
         <x:v>QA</x:v>
       </x:c>
-      <x:c r="D15" s="22" t="n">
+      <x:c r="D15" s="23" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E15" s="22" t="n">
+      <x:c r="E15" s="23" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="F15" s="22" t="n">
+      <x:c r="F15" s="23" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="G15" s="18" t="str">
         <x:v>En cours</x:v>
       </x:c>
-      <x:c r="H15" s="18" t="n">
+      <x:c r="H15" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$E$9:$E$38)=30,SUMIFS('Estimations'!$E$9:$E$38,'Estimations'!$B$9:$B$38,A15),NA())</x:f>
         <x:v>14</x:v>
       </x:c>
-      <x:c r="I15" s="18" t="n">
+      <x:c r="I15" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$F$9:$F$38)=30,SUMIFS('Estimations'!$F$9:$F$38,'Estimations'!$B$9:$B$38,A15),NA())</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="J15" s="18" t="n">
+      <x:c r="J15" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$G$9:$G$38)=30,SUMIFS('Estimations'!$G$9:$G$38,'Estimations'!$B$9:$B$38,A15),NA())</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="K15" s="2" t="n">
@@ -1611,10 +1839,10 @@
         <x:f>K15-H15</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="M15" s="20" t="str">
+      <x:c r="M15" s="21" t="str">
         <x:v>T02, T05</x:v>
       </x:c>
-      <x:c r="N15" s="20" t="n">
+      <x:c r="N15" s="21" t="n">
         <x:f>F15-E15</x:f>
         <x:v>1</x:v>
       </x:c>
@@ -1629,25 +1857,28 @@
       <x:c r="C16" s="2" t="str">
         <x:v>CP</x:v>
       </x:c>
-      <x:c r="D16" s="22" t="n">
+      <x:c r="D16" s="23" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E16" s="22" t="n">
+      <x:c r="E16" s="23" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="F16" s="22" t="n">
+      <x:c r="F16" s="23" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="G16" s="18" t="str">
         <x:v>En cours</x:v>
       </x:c>
-      <x:c r="H16" s="18" t="n">
+      <x:c r="H16" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$E$9:$E$38)=30,SUMIFS('Estimations'!$E$9:$E$38,'Estimations'!$B$9:$B$38,A16),NA())</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="I16" s="18" t="n">
+      <x:c r="I16" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$F$9:$F$38)=30,SUMIFS('Estimations'!$F$9:$F$38,'Estimations'!$B$9:$B$38,A16),NA())</x:f>
         <x:v>6</x:v>
       </x:c>
-      <x:c r="J16" s="18" t="n">
+      <x:c r="J16" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$G$9:$G$38)=30,SUMIFS('Estimations'!$G$9:$G$38,'Estimations'!$B$9:$B$38,A16),NA())</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="K16" s="2" t="n">
@@ -1658,10 +1889,10 @@
         <x:f>K16-H16</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M16" s="20" t="str">
+      <x:c r="M16" s="21" t="str">
         <x:v>Aucun</x:v>
       </x:c>
-      <x:c r="N16" s="20" t="n">
+      <x:c r="N16" s="21" t="n">
         <x:f>F16-E16</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1676,25 +1907,28 @@
       <x:c r="C17" s="2" t="str">
         <x:v>CP</x:v>
       </x:c>
-      <x:c r="D17" s="22" t="n">
+      <x:c r="D17" s="23" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="E17" s="22" t="n">
+      <x:c r="E17" s="23" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F17" s="22" t="n">
+      <x:c r="F17" s="23" t="n">
         <x:v>15</x:v>
       </x:c>
       <x:c r="G17" s="18" t="str">
         <x:v>À faire</x:v>
       </x:c>
-      <x:c r="H17" s="18" t="n">
+      <x:c r="H17" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$E$9:$E$38)=30,SUMIFS('Estimations'!$E$9:$E$38,'Estimations'!$B$9:$B$38,A17),NA())</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="I17" s="18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J17" s="18" t="n">
+      <x:c r="I17" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$F$9:$F$38)=30,SUMIFS('Estimations'!$F$9:$F$38,'Estimations'!$B$9:$B$38,A17),NA())</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J17" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$G$9:$G$38)=30,SUMIFS('Estimations'!$G$9:$G$38,'Estimations'!$B$9:$B$38,A17),NA())</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="K17" s="2" t="n">
@@ -1705,10 +1939,10 @@
         <x:f>K17-H17</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M17" s="20" t="str">
+      <x:c r="M17" s="21" t="str">
         <x:v>T07</x:v>
       </x:c>
-      <x:c r="N17" s="20" t="n">
+      <x:c r="N17" s="21" t="n">
         <x:f>F17-E17</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1723,25 +1957,28 @@
       <x:c r="C18" s="2" t="str">
         <x:v>DEV</x:v>
       </x:c>
-      <x:c r="D18" s="22" t="n">
+      <x:c r="D18" s="23" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="E18" s="22" t="n">
+      <x:c r="E18" s="23" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="F18" s="22" t="n">
+      <x:c r="F18" s="23" t="n">
         <x:v>14</x:v>
       </x:c>
       <x:c r="G18" s="18" t="str">
         <x:v>À faire</x:v>
       </x:c>
-      <x:c r="H18" s="18" t="n">
+      <x:c r="H18" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$E$9:$E$38)=30,SUMIFS('Estimations'!$E$9:$E$38,'Estimations'!$B$9:$B$38,A18),NA())</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="I18" s="18" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J18" s="18" t="n">
+      <x:c r="I18" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$F$9:$F$38)=30,SUMIFS('Estimations'!$F$9:$F$38,'Estimations'!$B$9:$B$38,A18),NA())</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J18" s="10" t="n">
+        <x:f>IF(COUNT('Estimations'!$G$9:$G$38)=30,SUMIFS('Estimations'!$G$9:$G$38,'Estimations'!$B$9:$B$38,A18),NA())</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="K18" s="2" t="n">
@@ -1752,10 +1989,10 @@
         <x:f>K18-H18</x:f>
         <x:v>-2</x:v>
       </x:c>
-      <x:c r="M18" s="20" t="str">
+      <x:c r="M18" s="21" t="str">
         <x:v>T06</x:v>
       </x:c>
-      <x:c r="N18" s="20" t="n">
+      <x:c r="N18" s="21" t="n">
         <x:f>F18-E18</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1779,7 +2016,7 @@
     <x:row r="20" ht="25" customHeight="1">
       <x:c r="A20" s="2"/>
       <x:c r="B20" s="2" t="str">
-        <x:v>Source : simulation pédagogique du lot. J1 à J15 ne sont pas des dates de réalisation historiques.</x:v>
+        <x:v>Charges calculées depuis les 30 activités de la feuille Estimations. Modifier cette feuille source.</x:v>
       </x:c>
       <x:c r="C20" s="2"/>
       <x:c r="D20" s="2"/>
@@ -1814,12 +2051,12 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="L9:L18">
-    <x:cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
+    <x:cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
       <x:formula>0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="N9:N18">
-    <x:cfRule type="cellIs" dxfId="3" priority="2" operator="greaterThan">
+    <x:cfRule type="cellIs" dxfId="4" priority="2" operator="greaterThan">
       <x:formula>0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -1945,7 +2182,7 @@
       <x:c r="A9" s="2" t="str">
         <x:v>R01</x:v>
       </x:c>
-      <x:c r="B9" s="23" t="str">
+      <x:c r="B9" s="25" t="str">
         <x:v>Environnement de démonstration indisponible</x:v>
       </x:c>
       <x:c r="C9" s="18" t="n">
@@ -1961,10 +2198,10 @@
       <x:c r="F9" s="2" t="str">
         <x:v>CP</x:v>
       </x:c>
-      <x:c r="G9" s="23" t="str">
+      <x:c r="G9" s="25" t="str">
         <x:v>Tester l'installation à J12, répéter à J14 et conserver des captures datées de secours</x:v>
       </x:c>
-      <x:c r="H9" s="23" t="str">
+      <x:c r="H9" s="25" t="str">
         <x:v>Sonde de santé indisponible ou base inaccessible</x:v>
       </x:c>
     </x:row>
@@ -1972,7 +2209,7 @@
       <x:c r="A10" s="2" t="str">
         <x:v>R02</x:v>
       </x:c>
-      <x:c r="B10" s="23" t="str">
+      <x:c r="B10" s="25" t="str">
         <x:v>Surcharge du chef de projet</x:v>
       </x:c>
       <x:c r="C10" s="18" t="n">
@@ -1988,10 +2225,10 @@
       <x:c r="F10" s="2" t="str">
         <x:v>CP</x:v>
       </x:c>
-      <x:c r="G10" s="23" t="str">
+      <x:c r="G10" s="25" t="str">
         <x:v>Limiter le travail simultané et faire préparer la grille de recette par QA</x:v>
       </x:c>
-      <x:c r="H10" s="23" t="str">
+      <x:c r="H10" s="25" t="str">
         <x:v>Prévision de charge supérieure à 90 % de la capacité</x:v>
       </x:c>
     </x:row>
@@ -1999,7 +2236,7 @@
       <x:c r="A11" s="2" t="str">
         <x:v>R03</x:v>
       </x:c>
-      <x:c r="B11" s="23" t="str">
+      <x:c r="B11" s="25" t="str">
         <x:v>Ajout tardif de contributions aux topos</x:v>
       </x:c>
       <x:c r="C11" s="18" t="n">
@@ -2015,10 +2252,10 @@
       <x:c r="F11" s="2" t="str">
         <x:v>CP</x:v>
       </x:c>
-      <x:c r="G11" s="23" t="str">
+      <x:c r="G11" s="25" t="str">
         <x:v>Reporter ce lot après la démonstration et consigner la décision client simulée</x:v>
       </x:c>
-      <x:c r="H11" s="23" t="str">
+      <x:c r="H11" s="25" t="str">
         <x:v>Nouvelle demande sans capacité ni recette disponible</x:v>
       </x:c>
     </x:row>
@@ -2026,7 +2263,7 @@
       <x:c r="A12" s="2" t="str">
         <x:v>R04</x:v>
       </x:c>
-      <x:c r="B12" s="23" t="str">
+      <x:c r="B12" s="25" t="str">
         <x:v>Défaut de capacité des événements</x:v>
       </x:c>
       <x:c r="C12" s="18" t="n">
@@ -2042,10 +2279,10 @@
       <x:c r="F12" s="2" t="str">
         <x:v>DEV</x:v>
       </x:c>
-      <x:c r="G12" s="23" t="str">
+      <x:c r="G12" s="25" t="str">
         <x:v>Vérifier l'inscription concurrente et les refus d'accès</x:v>
       </x:c>
-      <x:c r="H12" s="23" t="str">
+      <x:c r="H12" s="25" t="str">
         <x:v>Deux inscriptions acceptées sur la dernière place</x:v>
       </x:c>
     </x:row>
@@ -2053,7 +2290,7 @@
       <x:c r="A13" s="2" t="str">
         <x:v>R05</x:v>
       </x:c>
-      <x:c r="B13" s="23" t="str">
+      <x:c r="B13" s="25" t="str">
         <x:v>Consignes de dépôt non confirmées</x:v>
       </x:c>
       <x:c r="C13" s="18" t="n">
@@ -2069,10 +2306,10 @@
       <x:c r="F13" s="2" t="str">
         <x:v>CP</x:v>
       </x:c>
-      <x:c r="G13" s="23" t="str">
+      <x:c r="G13" s="25" t="str">
         <x:v>Consulter la convocation et le règlement spécial avant le dépôt</x:v>
       </x:c>
-      <x:c r="H13" s="23" t="str">
+      <x:c r="H13" s="25" t="str">
         <x:v>Date limite ou livrable demandé non identifié</x:v>
       </x:c>
     </x:row>
@@ -2100,7 +2337,7 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E9:E13">
-    <x:cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThanOrEqual">
+    <x:cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThanOrEqual">
       <x:formula>6</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -2112,4 +2349,1711 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="55" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2" ht="34" customHeight="1">
+      <x:c r="A2" s="2"/>
+      <x:c r="B2" s="3" t="str">
+        <x:v>Spity - Détail des estimations</x:v>
+      </x:c>
+      <x:c r="C2" s="2"/>
+      <x:c r="D2" s="2"/>
+      <x:c r="E2" s="2"/>
+      <x:c r="F2" s="2"/>
+      <x:c r="G2" s="2"/>
+      <x:c r="H2" s="2"/>
+      <x:c r="I2" s="2"/>
+    </x:row>
+    <x:row r="3" ht="25" customHeight="1">
+      <x:c r="A3" s="2"/>
+      <x:c r="B3" s="2"/>
+      <x:c r="C3" s="2"/>
+      <x:c r="D3" s="2"/>
+      <x:c r="E3" s="2"/>
+      <x:c r="F3" s="2"/>
+      <x:c r="G3" s="2"/>
+      <x:c r="H3" s="2"/>
+      <x:c r="I3" s="2"/>
+    </x:row>
+    <x:row r="4" ht="25" customHeight="1">
+      <x:c r="A4" s="2"/>
+      <x:c r="B4" s="4" t="str">
+        <x:v>SIMULATION PÉDAGOGIQUE - état à J10, horizon de 15 jours ouvrés</x:v>
+      </x:c>
+      <x:c r="C4" s="2"/>
+      <x:c r="D4" s="2"/>
+      <x:c r="E4" s="2"/>
+      <x:c r="F4" s="2"/>
+      <x:c r="G4" s="2"/>
+      <x:c r="H4" s="2"/>
+      <x:c r="I4" s="2"/>
+    </x:row>
+    <x:row r="5" ht="25" customHeight="1">
+      <x:c r="A5" s="2"/>
+      <x:c r="B5" s="4" t="str">
+        <x:v>Les jours, charges, taux et réunions du cas ne sont pas des observations historiques.</x:v>
+      </x:c>
+      <x:c r="C5" s="2"/>
+      <x:c r="D5" s="2"/>
+      <x:c r="E5" s="2"/>
+      <x:c r="F5" s="2"/>
+      <x:c r="G5" s="2"/>
+      <x:c r="H5" s="2"/>
+      <x:c r="I5" s="2"/>
+    </x:row>
+    <x:row r="6" ht="25" customHeight="1">
+      <x:c r="A6" s="2"/>
+      <x:c r="B6" s="2"/>
+      <x:c r="C6" s="2"/>
+      <x:c r="D6" s="2"/>
+      <x:c r="E6" s="2"/>
+      <x:c r="F6" s="2"/>
+      <x:c r="G6" s="2"/>
+      <x:c r="H6" s="2"/>
+      <x:c r="I6" s="2"/>
+    </x:row>
+    <x:row r="7" ht="25" customHeight="1">
+      <x:c r="A7" s="2"/>
+      <x:c r="B7" s="2"/>
+      <x:c r="C7" s="2"/>
+      <x:c r="D7" s="2"/>
+      <x:c r="E7" s="2"/>
+      <x:c r="F7" s="2"/>
+      <x:c r="G7" s="2"/>
+      <x:c r="H7" s="2"/>
+      <x:c r="I7" s="2"/>
+    </x:row>
+    <x:row r="8" ht="36" customHeight="1">
+      <x:c r="A8" s="7" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="str">
+        <x:v>Tâche</x:v>
+      </x:c>
+      <x:c r="C8" s="7" t="str">
+        <x:v>Rôle</x:v>
+      </x:c>
+      <x:c r="D8" s="7" t="str">
+        <x:v>Activité du scénario</x:v>
+      </x:c>
+      <x:c r="E8" s="7" t="str">
+        <x:v>Prévu h</x:v>
+      </x:c>
+      <x:c r="F8" s="7" t="str">
+        <x:v>Consommé h</x:v>
+      </x:c>
+      <x:c r="G8" s="7" t="str">
+        <x:v>Restant h</x:v>
+      </x:c>
+      <x:c r="H8" s="7" t="str">
+        <x:v>Prévision h</x:v>
+      </x:c>
+      <x:c r="I8" s="7" t="str">
+        <x:v>Écart h</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="25" customHeight="1">
+      <x:c r="A9" s="2" t="str">
+        <x:v>T01.1</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="str">
+        <x:v>T01</x:v>
+      </x:c>
+      <x:c r="C9" s="2" t="str">
+        <x:v>CP</x:v>
+      </x:c>
+      <x:c r="D9" s="2" t="str">
+        <x:v>Cadrer les deux parcours</x:v>
+      </x:c>
+      <x:c r="E9" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F9" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G9" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="2" t="n">
+        <x:f>IF(COUNT(F9:G9)=2,SUM(F9:G9),NA())</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I9" s="2" t="n">
+        <x:f>H9-E9</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="25" customHeight="1">
+      <x:c r="A10" s="2" t="str">
+        <x:v>T01.2</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="str">
+        <x:v>T01</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
+        <x:v>CP</x:v>
+      </x:c>
+      <x:c r="D10" s="2" t="str">
+        <x:v>Fixer inclusions et exclusions</x:v>
+      </x:c>
+      <x:c r="E10" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F10" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G10" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H10" s="2" t="n">
+        <x:f>IF(COUNT(F10:G10)=2,SUM(F10:G10),NA())</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I10" s="2" t="n">
+        <x:f>H10-E10</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="25" customHeight="1">
+      <x:c r="A11" s="2" t="str">
+        <x:v>T01.3</x:v>
+      </x:c>
+      <x:c r="B11" s="2" t="str">
+        <x:v>T01</x:v>
+      </x:c>
+      <x:c r="C11" s="2" t="str">
+        <x:v>CP</x:v>
+      </x:c>
+      <x:c r="D11" s="2" t="str">
+        <x:v>Préparer les critères de décision</x:v>
+      </x:c>
+      <x:c r="E11" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F11" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G11" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H11" s="2" t="n">
+        <x:f>IF(COUNT(F11:G11)=2,SUM(F11:G11),NA())</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I11" s="2" t="n">
+        <x:f>H11-E11</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="25" customHeight="1">
+      <x:c r="A12" s="2" t="str">
+        <x:v>T02.1</x:v>
+      </x:c>
+      <x:c r="B12" s="2" t="str">
+        <x:v>T02</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="D12" s="2" t="str">
+        <x:v>Écrire les cas grimpeur</x:v>
+      </x:c>
+      <x:c r="E12" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F12" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G12" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H12" s="2" t="n">
+        <x:f>IF(COUNT(F12:G12)=2,SUM(F12:G12),NA())</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I12" s="2" t="n">
+        <x:f>H12-E12</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="25" customHeight="1">
+      <x:c r="A13" s="2" t="str">
+        <x:v>T02.2</x:v>
+      </x:c>
+      <x:c r="B13" s="2" t="str">
+        <x:v>T02</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="D13" s="2" t="str">
+        <x:v>Écrire les cas club</x:v>
+      </x:c>
+      <x:c r="E13" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F13" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G13" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H13" s="2" t="n">
+        <x:f>IF(COUNT(F13:G13)=2,SUM(F13:G13),NA())</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I13" s="2" t="n">
+        <x:f>H13-E13</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="25" customHeight="1">
+      <x:c r="A14" s="2" t="str">
+        <x:v>T02.3</x:v>
+      </x:c>
+      <x:c r="B14" s="2" t="str">
+        <x:v>T02</x:v>
+      </x:c>
+      <x:c r="C14" s="2" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="D14" s="2" t="str">
+        <x:v>Définir les critères accessibles</x:v>
+      </x:c>
+      <x:c r="E14" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F14" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G14" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H14" s="2" t="n">
+        <x:f>IF(COUNT(F14:G14)=2,SUM(F14:G14),NA())</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I14" s="2" t="n">
+        <x:f>H14-E14</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="25" customHeight="1">
+      <x:c r="A15" s="2" t="str">
+        <x:v>T03.1</x:v>
+      </x:c>
+      <x:c r="B15" s="2" t="str">
+        <x:v>T03</x:v>
+      </x:c>
+      <x:c r="C15" s="2" t="str">
+        <x:v>CP</x:v>
+      </x:c>
+      <x:c r="D15" s="2" t="str">
+        <x:v>Décomposer le lot</x:v>
+      </x:c>
+      <x:c r="E15" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F15" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G15" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H15" s="2" t="n">
+        <x:f>IF(COUNT(F15:G15)=2,SUM(F15:G15),NA())</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I15" s="2" t="n">
+        <x:f>H15-E15</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="25" customHeight="1">
+      <x:c r="A16" s="2" t="str">
+        <x:v>T03.2</x:v>
+      </x:c>
+      <x:c r="B16" s="2" t="str">
+        <x:v>T03</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="str">
+        <x:v>CP</x:v>
+      </x:c>
+      <x:c r="D16" s="2" t="str">
+        <x:v>Ajuster les dépendances de recette</x:v>
+      </x:c>
+      <x:c r="E16" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F16" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G16" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H16" s="2" t="n">
+        <x:f>IF(COUNT(F16:G16)=2,SUM(F16:G16),NA())</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I16" s="2" t="n">
+        <x:f>H16-E16</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="25" customHeight="1">
+      <x:c r="A17" s="2" t="str">
+        <x:v>T03.3</x:v>
+      </x:c>
+      <x:c r="B17" s="2" t="str">
+        <x:v>T03</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
+        <x:v>CP</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="str">
+        <x:v>Affecter les responsabilités</x:v>
+      </x:c>
+      <x:c r="E17" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F17" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G17" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H17" s="2" t="n">
+        <x:f>IF(COUNT(F17:G17)=2,SUM(F17:G17),NA())</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I17" s="2" t="n">
+        <x:f>H17-E17</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="25" customHeight="1">
+      <x:c r="A18" s="2" t="str">
+        <x:v>T04.1</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="str">
+        <x:v>T04</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
+        <x:v>DEV</x:v>
+      </x:c>
+      <x:c r="D18" s="2" t="str">
+        <x:v>Vérifier les contrats accès et profils</x:v>
+      </x:c>
+      <x:c r="E18" s="18" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F18" s="18" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G18" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H18" s="2" t="n">
+        <x:f>IF(COUNT(F18:G18)=2,SUM(F18:G18),NA())</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I18" s="2" t="n">
+        <x:f>H18-E18</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="25" customHeight="1">
+      <x:c r="A19" s="2" t="str">
+        <x:v>T04.2</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="str">
+        <x:v>T04</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
+        <x:v>DEV</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="str">
+        <x:v>Stabiliser les contrôles de rôles</x:v>
+      </x:c>
+      <x:c r="E19" s="18" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F19" s="18" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="G19" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H19" s="2" t="n">
+        <x:f>IF(COUNT(F19:G19)=2,SUM(F19:G19),NA())</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="I19" s="2" t="n">
+        <x:f>H19-E19</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="25" customHeight="1">
+      <x:c r="A20" s="2" t="str">
+        <x:v>T04.3</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="str">
+        <x:v>T04</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
+        <x:v>DEV</x:v>
+      </x:c>
+      <x:c r="D20" s="2" t="str">
+        <x:v>Rejouer les cas de session et profil</x:v>
+      </x:c>
+      <x:c r="E20" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F20" s="18" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G20" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H20" s="2" t="n">
+        <x:f>IF(COUNT(F20:G20)=2,SUM(F20:G20),NA())</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I20" s="2" t="n">
+        <x:f>H20-E20</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="25" customHeight="1">
+      <x:c r="A21" s="2" t="str">
+        <x:v>T05.1</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="str">
+        <x:v>T05</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
+        <x:v>DEV</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="str">
+        <x:v>Préparer les cas de compatibilité</x:v>
+      </x:c>
+      <x:c r="E21" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F21" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G21" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H21" s="2" t="n">
+        <x:f>IF(COUNT(F21:G21)=2,SUM(F21:G21),NA())</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I21" s="2" t="n">
+        <x:f>H21-E21</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="25" customHeight="1">
+      <x:c r="A22" s="2" t="str">
+        <x:v>T05.2</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="str">
+        <x:v>T05</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
+        <x:v>DEV</x:v>
+      </x:c>
+      <x:c r="D22" s="2" t="str">
+        <x:v>Stabiliser filtres et demande partenaire</x:v>
+      </x:c>
+      <x:c r="E22" s="18" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F22" s="18" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="G22" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H22" s="2" t="n">
+        <x:f>IF(COUNT(F22:G22)=2,SUM(F22:G22),NA())</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I22" s="2" t="n">
+        <x:f>H22-E22</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="25" customHeight="1">
+      <x:c r="A23" s="2" t="str">
+        <x:v>T05.3</x:v>
+      </x:c>
+      <x:c r="B23" s="2" t="str">
+        <x:v>T05</x:v>
+      </x:c>
+      <x:c r="C23" s="2" t="str">
+        <x:v>DEV</x:v>
+      </x:c>
+      <x:c r="D23" s="2" t="str">
+        <x:v>Vérifier le parcours partenaire</x:v>
+      </x:c>
+      <x:c r="E23" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F23" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G23" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H23" s="2" t="n">
+        <x:f>IF(COUNT(F23:G23)=2,SUM(F23:G23),NA())</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I23" s="2" t="n">
+        <x:f>H23-E23</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="25" customHeight="1">
+      <x:c r="A24" s="2" t="str">
+        <x:v>T06.1</x:v>
+      </x:c>
+      <x:c r="B24" s="2" t="str">
+        <x:v>T06</x:v>
+      </x:c>
+      <x:c r="C24" s="2" t="str">
+        <x:v>DEV</x:v>
+      </x:c>
+      <x:c r="D24" s="2" t="str">
+        <x:v>Préparer les règles événement</x:v>
+      </x:c>
+      <x:c r="E24" s="18" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F24" s="18" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G24" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H24" s="2" t="n">
+        <x:f>IF(COUNT(F24:G24)=2,SUM(F24:G24),NA())</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="I24" s="2" t="n">
+        <x:f>H24-E24</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="25" customHeight="1">
+      <x:c r="A25" s="2" t="str">
+        <x:v>T06.2</x:v>
+      </x:c>
+      <x:c r="B25" s="2" t="str">
+        <x:v>T06</x:v>
+      </x:c>
+      <x:c r="C25" s="2" t="str">
+        <x:v>DEV</x:v>
+      </x:c>
+      <x:c r="D25" s="2" t="str">
+        <x:v>Stabiliser capacité et inscriptions</x:v>
+      </x:c>
+      <x:c r="E25" s="18" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F25" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G25" s="18" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H25" s="2" t="n">
+        <x:f>IF(COUNT(F25:G25)=2,SUM(F25:G25),NA())</x:f>
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I25" s="2" t="n">
+        <x:f>H25-E25</x:f>
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="25" customHeight="1">
+      <x:c r="A26" s="2" t="str">
+        <x:v>T06.3</x:v>
+      </x:c>
+      <x:c r="B26" s="2" t="str">
+        <x:v>T06</x:v>
+      </x:c>
+      <x:c r="C26" s="2" t="str">
+        <x:v>DEV</x:v>
+      </x:c>
+      <x:c r="D26" s="2" t="str">
+        <x:v>Contrôler les participants autorisés</x:v>
+      </x:c>
+      <x:c r="E26" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F26" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G26" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H26" s="2" t="n">
+        <x:f>IF(COUNT(F26:G26)=2,SUM(F26:G26),NA())</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I26" s="2" t="n">
+        <x:f>H26-E26</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="25" customHeight="1">
+      <x:c r="A27" s="2" t="str">
+        <x:v>T07.1</x:v>
+      </x:c>
+      <x:c r="B27" s="2" t="str">
+        <x:v>T07</x:v>
+      </x:c>
+      <x:c r="C27" s="2" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="D27" s="2" t="str">
+        <x:v>Préparer jeux de données et recette</x:v>
+      </x:c>
+      <x:c r="E27" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F27" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G27" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H27" s="2" t="n">
+        <x:f>IF(COUNT(F27:G27)=2,SUM(F27:G27),NA())</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="I27" s="2" t="n">
+        <x:f>H27-E27</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="25" customHeight="1">
+      <x:c r="A28" s="2" t="str">
+        <x:v>T07.2</x:v>
+      </x:c>
+      <x:c r="B28" s="2" t="str">
+        <x:v>T07</x:v>
+      </x:c>
+      <x:c r="C28" s="2" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="D28" s="2" t="str">
+        <x:v>Rejouer les parcours et les limites</x:v>
+      </x:c>
+      <x:c r="E28" s="18" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F28" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G28" s="18" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H28" s="2" t="n">
+        <x:f>IF(COUNT(F28:G28)=2,SUM(F28:G28),NA())</x:f>
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I28" s="2" t="n">
+        <x:f>H28-E28</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="25" customHeight="1">
+      <x:c r="A29" s="2" t="str">
+        <x:v>T07.3</x:v>
+      </x:c>
+      <x:c r="B29" s="2" t="str">
+        <x:v>T07</x:v>
+      </x:c>
+      <x:c r="C29" s="2" t="str">
+        <x:v>QA</x:v>
+      </x:c>
+      <x:c r="D29" s="2" t="str">
+        <x:v>Contrôler clavier, erreurs et retours</x:v>
+      </x:c>
+      <x:c r="E29" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F29" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G29" s="18" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H29" s="2" t="n">
+        <x:f>IF(COUNT(F29:G29)=2,SUM(F29:G29),NA())</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I29" s="2" t="n">
+        <x:f>H29-E29</x:f>
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="25" customHeight="1">
+      <x:c r="A30" s="2" t="str">
+        <x:v>T08.1</x:v>
+      </x:c>
+      <x:c r="B30" s="2" t="str">
+        <x:v>T08</x:v>
+      </x:c>
+      <x:c r="C30" s="2" t="str">
+        <x:v>CP</x:v>
+      </x:c>
+      <x:c r="D30" s="2" t="str">
+        <x:v>Suivre charges et dépendances</x:v>
+      </x:c>
+      <x:c r="E30" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F30" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G30" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H30" s="2" t="n">
+        <x:f>IF(COUNT(F30:G30)=2,SUM(F30:G30),NA())</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I30" s="2" t="n">
+        <x:f>H30-E30</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="25" customHeight="1">
+      <x:c r="A31" s="2" t="str">
+        <x:v>T08.2</x:v>
+      </x:c>
+      <x:c r="B31" s="2" t="str">
+        <x:v>T08</x:v>
+      </x:c>
+      <x:c r="C31" s="2" t="str">
+        <x:v>CP</x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="str">
+        <x:v>Préparer la revue et arbitrer</x:v>
+      </x:c>
+      <x:c r="E31" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F31" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G31" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H31" s="2" t="n">
+        <x:f>IF(COUNT(F31:G31)=2,SUM(F31:G31),NA())</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I31" s="2" t="n">
+        <x:f>H31-E31</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="25" customHeight="1">
+      <x:c r="A32" s="2" t="str">
+        <x:v>T08.3</x:v>
+      </x:c>
+      <x:c r="B32" s="2" t="str">
+        <x:v>T08</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="str">
+        <x:v>CP</x:v>
+      </x:c>
+      <x:c r="D32" s="2" t="str">
+        <x:v>Formaliser réserves et validation</x:v>
+      </x:c>
+      <x:c r="E32" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F32" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G32" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H32" s="2" t="n">
+        <x:f>IF(COUNT(F32:G32)=2,SUM(F32:G32),NA())</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I32" s="2" t="n">
+        <x:f>H32-E32</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="25" customHeight="1">
+      <x:c r="A33" s="2" t="str">
+        <x:v>T09.1</x:v>
+      </x:c>
+      <x:c r="B33" s="2" t="str">
+        <x:v>T09</x:v>
+      </x:c>
+      <x:c r="C33" s="2" t="str">
+        <x:v>CP</x:v>
+      </x:c>
+      <x:c r="D33" s="2" t="str">
+        <x:v>Construire le support de restitution</x:v>
+      </x:c>
+      <x:c r="E33" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F33" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G33" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H33" s="2" t="n">
+        <x:f>IF(COUNT(F33:G33)=2,SUM(F33:G33),NA())</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I33" s="2" t="n">
+        <x:f>H33-E33</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="25" customHeight="1">
+      <x:c r="A34" s="2" t="str">
+        <x:v>T09.2</x:v>
+      </x:c>
+      <x:c r="B34" s="2" t="str">
+        <x:v>T09</x:v>
+      </x:c>
+      <x:c r="C34" s="2" t="str">
+        <x:v>CP</x:v>
+      </x:c>
+      <x:c r="D34" s="2" t="str">
+        <x:v>Répéter le parcours et les secours</x:v>
+      </x:c>
+      <x:c r="E34" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F34" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G34" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H34" s="2" t="n">
+        <x:f>IF(COUNT(F34:G34)=2,SUM(F34:G34),NA())</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I34" s="2" t="n">
+        <x:f>H34-E34</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="25" customHeight="1">
+      <x:c r="A35" s="2" t="str">
+        <x:v>T09.3</x:v>
+      </x:c>
+      <x:c r="B35" s="2" t="str">
+        <x:v>T09</x:v>
+      </x:c>
+      <x:c r="C35" s="2" t="str">
+        <x:v>CP</x:v>
+      </x:c>
+      <x:c r="D35" s="2" t="str">
+        <x:v>Préparer la transmission maintenance</x:v>
+      </x:c>
+      <x:c r="E35" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F35" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G35" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H35" s="2" t="n">
+        <x:f>IF(COUNT(F35:G35)=2,SUM(F35:G35),NA())</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I35" s="2" t="n">
+        <x:f>H35-E35</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="25" customHeight="1">
+      <x:c r="A36" s="2" t="str">
+        <x:v>T10.1</x:v>
+      </x:c>
+      <x:c r="B36" s="2" t="str">
+        <x:v>T10</x:v>
+      </x:c>
+      <x:c r="C36" s="2" t="str">
+        <x:v>DEV</x:v>
+      </x:c>
+      <x:c r="D36" s="2" t="str">
+        <x:v>Corriger les défauts bloquants du cas</x:v>
+      </x:c>
+      <x:c r="E36" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F36" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G36" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H36" s="2" t="n">
+        <x:f>IF(COUNT(F36:G36)=2,SUM(F36:G36),NA())</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I36" s="2" t="n">
+        <x:f>H36-E36</x:f>
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="25" customHeight="1">
+      <x:c r="A37" s="2" t="str">
+        <x:v>T10.2</x:v>
+      </x:c>
+      <x:c r="B37" s="2" t="str">
+        <x:v>T10</x:v>
+      </x:c>
+      <x:c r="C37" s="2" t="str">
+        <x:v>DEV</x:v>
+      </x:c>
+      <x:c r="D37" s="2" t="str">
+        <x:v>Rejouer les tests de non-régression</x:v>
+      </x:c>
+      <x:c r="E37" s="18" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F37" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G37" s="18" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H37" s="2" t="n">
+        <x:f>IF(COUNT(F37:G37)=2,SUM(F37:G37),NA())</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="I37" s="2" t="n">
+        <x:f>H37-E37</x:f>
+        <x:v>-1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="25" customHeight="1">
+      <x:c r="A38" s="2" t="str">
+        <x:v>T10.3</x:v>
+      </x:c>
+      <x:c r="B38" s="2" t="str">
+        <x:v>T10</x:v>
+      </x:c>
+      <x:c r="C38" s="2" t="str">
+        <x:v>DEV</x:v>
+      </x:c>
+      <x:c r="D38" s="2" t="str">
+        <x:v>Documenter les réserves</x:v>
+      </x:c>
+      <x:c r="E38" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F38" s="18" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G38" s="18" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H38" s="2" t="n">
+        <x:f>IF(COUNT(F38:G38)=2,SUM(F38:G38),NA())</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I38" s="2" t="n">
+        <x:f>H38-E38</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="25" customHeight="1">
+      <x:c r="A39" s="2"/>
+      <x:c r="B39" s="2"/>
+      <x:c r="C39" s="2"/>
+      <x:c r="D39" s="2"/>
+      <x:c r="E39" s="2"/>
+      <x:c r="F39" s="2"/>
+      <x:c r="G39" s="2"/>
+      <x:c r="H39" s="2"/>
+      <x:c r="I39" s="2"/>
+    </x:row>
+    <x:row r="40" ht="25" customHeight="1">
+      <x:c r="A40" s="2"/>
+      <x:c r="B40" s="2" t="str">
+        <x:v>Source : hypothèses du cas, donnees/pilotage.json et A09. Une ligne décrit un livrable.</x:v>
+      </x:c>
+      <x:c r="C40" s="2"/>
+      <x:c r="D40" s="2"/>
+      <x:c r="E40" s="2"/>
+      <x:c r="F40" s="2"/>
+      <x:c r="G40" s="2"/>
+      <x:c r="H40" s="2"/>
+      <x:c r="I40" s="2"/>
+    </x:row>
+    <x:row r="41" ht="25" customHeight="1">
+      <x:c r="A41" s="2"/>
+      <x:c r="B41" s="2" t="str">
+        <x:v>La formation est incluse dans T03, T06 et T07. Les heures ne proviennent pas de Linear.</x:v>
+      </x:c>
+      <x:c r="C41" s="2"/>
+      <x:c r="D41" s="2"/>
+      <x:c r="E41" s="2"/>
+      <x:c r="F41" s="2"/>
+      <x:c r="G41" s="2"/>
+      <x:c r="H41" s="2"/>
+      <x:c r="I41" s="2"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="65" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="19" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="95" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="2" ht="25" customHeight="1">
+      <x:c r="A2" s="2"/>
+      <x:c r="B2" s="3" t="str">
+        <x:v>Spity - Relevé Linear du 14 septembre 2026</x:v>
+      </x:c>
+      <x:c r="C2" s="2"/>
+      <x:c r="D2" s="2"/>
+      <x:c r="E2" s="2"/>
+      <x:c r="F2" s="2"/>
+    </x:row>
+    <x:row r="3" ht="25" customHeight="1">
+      <x:c r="A3" s="2"/>
+      <x:c r="B3" s="2"/>
+      <x:c r="C3" s="2"/>
+      <x:c r="D3" s="2"/>
+      <x:c r="E3" s="2"/>
+      <x:c r="F3" s="2"/>
+    </x:row>
+    <x:row r="4" ht="25" customHeight="1">
+      <x:c r="A4" s="2"/>
+      <x:c r="B4" s="2" t="str">
+        <x:v>OBSERVATION : statuts lus dans le tableau authentifié. Estimations absentes de cette source.</x:v>
+      </x:c>
+      <x:c r="C4" s="2"/>
+      <x:c r="D4" s="2"/>
+      <x:c r="E4" s="2"/>
+      <x:c r="F4" s="2"/>
+    </x:row>
+    <x:row r="5" ht="25" customHeight="1">
+      <x:c r="A5" s="2"/>
+      <x:c r="B5" s="2" t="str">
+        <x:v>12 Done / 24 non annulés = 50 % des tickets, sans pondération par effort.</x:v>
+      </x:c>
+      <x:c r="C5" s="2"/>
+      <x:c r="D5" s="2"/>
+      <x:c r="E5" s="2"/>
+      <x:c r="F5" s="2"/>
+    </x:row>
+    <x:row r="6" ht="25" customHeight="1">
+      <x:c r="A6" s="2"/>
+      <x:c r="B6" s="2"/>
+      <x:c r="C6" s="2"/>
+      <x:c r="D6" s="2"/>
+      <x:c r="E6" s="2"/>
+      <x:c r="F6" s="2"/>
+    </x:row>
+    <x:row r="7" ht="25" customHeight="1">
+      <x:c r="A7" s="2"/>
+      <x:c r="B7" s="2"/>
+      <x:c r="C7" s="2"/>
+      <x:c r="D7" s="2"/>
+      <x:c r="E7" s="2"/>
+      <x:c r="F7" s="2"/>
+    </x:row>
+    <x:row r="8" ht="36" customHeight="1">
+      <x:c r="A8" s="7" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="str">
+        <x:v>Intitulé observé</x:v>
+      </x:c>
+      <x:c r="C8" s="7" t="str">
+        <x:v>Statut</x:v>
+      </x:c>
+      <x:c r="D8" s="7" t="str">
+        <x:v>Priorité</x:v>
+      </x:c>
+      <x:c r="E8" s="7" t="str">
+        <x:v>Affectation</x:v>
+      </x:c>
+      <x:c r="F8" s="7" t="str">
+        <x:v>Source URL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="39" customHeight="1">
+      <x:c r="A9" s="2" t="str">
+        <x:v>SPI-5</x:v>
+      </x:c>
+      <x:c r="B9" s="25" t="str">
+        <x:v>SPITY-001: Prisma schema User + Club</x:v>
+      </x:c>
+      <x:c r="C9" s="2" t="str">
+        <x:v>Canceled</x:v>
+      </x:c>
+      <x:c r="D9" s="2" t="str">
+        <x:v>Urgent</x:v>
+      </x:c>
+      <x:c r="E9" s="2" t="str">
+        <x:v>Non affecté</x:v>
+      </x:c>
+      <x:c r="F9" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-5/spity-001-prisma-schema-user-club</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="39" customHeight="1">
+      <x:c r="A10" s="2" t="str">
+        <x:v>SPI-6</x:v>
+      </x:c>
+      <x:c r="B10" s="25" t="str">
+        <x:v>SPITY-002: JWT auth grimpeur/club</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="str">
+        <x:v>Todo</x:v>
+      </x:c>
+      <x:c r="D10" s="2" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E10" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F10" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-6/spity-002-jwt-auth-grimpeurclub</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="39" customHeight="1">
+      <x:c r="A11" s="2" t="str">
+        <x:v>SPI-7</x:v>
+      </x:c>
+      <x:c r="B11" s="25" t="str">
+        <x:v>SPITY-003: Login/register pages</x:v>
+      </x:c>
+      <x:c r="C11" s="2" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D11" s="2" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E11" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F11" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-7/spity-003-loginregister-pages</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="39" customHeight="1">
+      <x:c r="A12" s="2" t="str">
+        <x:v>SPI-8</x:v>
+      </x:c>
+      <x:c r="B12" s="25" t="str">
+        <x:v>SPITY-004: Docker compose Next+MariaDB+phpMyAdmin</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D12" s="2" t="str">
+        <x:v>Urgent</x:v>
+      </x:c>
+      <x:c r="E12" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F12" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-8/spity-004-docker-compose-nextmariadbphpmyadmin</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="39" customHeight="1">
+      <x:c r="A13" s="2" t="str">
+        <x:v>SPI-9</x:v>
+      </x:c>
+      <x:c r="B13" s="25" t="str">
+        <x:v>SPITY-005: Drizzle schema initial</x:v>
+      </x:c>
+      <x:c r="C13" s="2" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D13" s="2" t="str">
+        <x:v>Urgent</x:v>
+      </x:c>
+      <x:c r="E13" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F13" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-9/spity-005-drizzle-schema-initial</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="39" customHeight="1">
+      <x:c r="A14" s="2" t="str">
+        <x:v>SPI-10</x:v>
+      </x:c>
+      <x:c r="B14" s="25" t="str">
+        <x:v>SPITY-006: GitHub Actions CI/CD</x:v>
+      </x:c>
+      <x:c r="C14" s="2" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D14" s="2" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E14" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F14" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-10/spity-006-github-actions-cicd</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="39" customHeight="1">
+      <x:c r="A15" s="2" t="str">
+        <x:v>SPI-11</x:v>
+      </x:c>
+      <x:c r="B15" s="25" t="str">
+        <x:v>SPITY-007: CRUD profil grimpeur (disciplines, niveaux, matos)</x:v>
+      </x:c>
+      <x:c r="C15" s="2" t="str">
+        <x:v>Todo</x:v>
+      </x:c>
+      <x:c r="D15" s="2" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E15" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F15" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-11/spity-007-crud-profil-grimpeur-disciplines-niveaux-matos</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="39" customHeight="1">
+      <x:c r="A16" s="2" t="str">
+        <x:v>SPI-12</x:v>
+      </x:c>
+      <x:c r="B16" s="25" t="str">
+        <x:v>SPITY-008: CRUD profil club (coachs, validation)</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D16" s="2" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E16" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F16" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-12/spity-008-crud-profil-club-coachs-validation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="39" customHeight="1">
+      <x:c r="A17" s="2" t="str">
+        <x:v>SPI-13</x:v>
+      </x:c>
+      <x:c r="B17" s="25" t="str">
+        <x:v>SPITY-009: Page profil grimpeur + édition</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E17" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F17" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-13/spity-009-page-profil-grimpeur-edition</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="39" customHeight="1">
+      <x:c r="A18" s="2" t="str">
+        <x:v>SPI-14</x:v>
+      </x:c>
+      <x:c r="B18" s="25" t="str">
+        <x:v>SPITY-010: Page profil club</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D18" s="2" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E18" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F18" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-14/spity-010-page-profil-club</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="39" customHeight="1">
+      <x:c r="A19" s="2" t="str">
+        <x:v>SPI-15</x:v>
+      </x:c>
+      <x:c r="B19" s="25" t="str">
+        <x:v>SPITY-011: CRUD Post (texte, media, tags, cotation)</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
+        <x:v>Todo</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F19" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-15/spity-011-crud-post-texte-media-tags-cotation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="39" customHeight="1">
+      <x:c r="A20" s="2" t="str">
+        <x:v>SPI-16</x:v>
+      </x:c>
+      <x:c r="B20" s="25" t="str">
+        <x:v>SPITY-012: Likes + commentaires</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D20" s="2" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E20" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F20" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-16/spity-012-likes-commentaires</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="39" customHeight="1">
+      <x:c r="A21" s="2" t="str">
+        <x:v>SPI-17</x:v>
+      </x:c>
+      <x:c r="B21" s="25" t="str">
+        <x:v>SPITY-013: Feed principal (posts + events épinglés)</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F21" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-17/spity-013-feed-principal-posts-events-epingles</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="39" customHeight="1">
+      <x:c r="A22" s="2" t="str">
+        <x:v>SPI-18</x:v>
+      </x:c>
+      <x:c r="B22" s="25" t="str">
+        <x:v>SPITY-014: Create post + upload images</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
+        <x:v>Todo</x:v>
+      </x:c>
+      <x:c r="D22" s="2" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E22" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F22" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-18/spity-014-create-post-upload-images</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="39" customHeight="1">
+      <x:c r="A23" s="2" t="str">
+        <x:v>SPI-19</x:v>
+      </x:c>
+      <x:c r="B23" s="25" t="str">
+        <x:v>SPITY-015: Modèles Salle/Falaise (géoloc)</x:v>
+      </x:c>
+      <x:c r="C23" s="2" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D23" s="2" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E23" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F23" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-19/spity-015-modeles-sallefalaise-geoloc</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="39" customHeight="1">
+      <x:c r="A24" s="2" t="str">
+        <x:v>SPI-20</x:v>
+      </x:c>
+      <x:c r="B24" s="25" t="str">
+        <x:v>SPITY-016: Modèle Voie + topos (cotation, état)</x:v>
+      </x:c>
+      <x:c r="C24" s="2" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D24" s="2" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E24" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F24" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-20/spity-016-modele-voie-topos-cotation-etat</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="39" customHeight="1">
+      <x:c r="A25" s="2" t="str">
+        <x:v>SPI-21</x:v>
+      </x:c>
+      <x:c r="B25" s="25" t="str">
+        <x:v>SPITY-017: Carte interactive salles/falaises/clubs</x:v>
+      </x:c>
+      <x:c r="C25" s="2" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D25" s="2" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E25" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F25" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-21/spity-017-carte-interactive-sallesfalaisesclubs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="39" customHeight="1">
+      <x:c r="A26" s="2" t="str">
+        <x:v>SPI-22</x:v>
+      </x:c>
+      <x:c r="B26" s="25" t="str">
+        <x:v>SPITY-018: Fiche falaise + topos collaboratifs</x:v>
+      </x:c>
+      <x:c r="C26" s="2" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D26" s="2" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E26" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F26" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-22/spity-018-fiche-falaise-topos-collaboratifs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="39" customHeight="1">
+      <x:c r="A27" s="2" t="str">
+        <x:v>SPI-23</x:v>
+      </x:c>
+      <x:c r="B27" s="25" t="str">
+        <x:v>SPITY-019: CRUD Event club (inscriptions, capacité)</x:v>
+      </x:c>
+      <x:c r="C27" s="2" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D27" s="2" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E27" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F27" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-23/spity-019-crud-event-club-inscriptions-capacite</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="39" customHeight="1">
+      <x:c r="A28" s="2" t="str">
+        <x:v>SPI-24</x:v>
+      </x:c>
+      <x:c r="B28" s="25" t="str">
+        <x:v>SPITY-020: Club dashboard (stats, events)</x:v>
+      </x:c>
+      <x:c r="C28" s="2" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D28" s="2" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E28" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F28" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-24/spity-020-club-dashboard-stats-events</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="39" customHeight="1">
+      <x:c r="A29" s="2" t="str">
+        <x:v>SPI-25</x:v>
+      </x:c>
+      <x:c r="B29" s="25" t="str">
+        <x:v>SPITY-021: Calendrier events + inscription</x:v>
+      </x:c>
+      <x:c r="C29" s="2" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D29" s="2" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E29" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F29" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-25/spity-021-calendrier-events-inscription</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="39" customHeight="1">
+      <x:c r="A30" s="2" t="str">
+        <x:v>SPI-26</x:v>
+      </x:c>
+      <x:c r="B30" s="25" t="str">
+        <x:v>SPITY-022: Club dashboard</x:v>
+      </x:c>
+      <x:c r="C30" s="2" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D30" s="2" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E30" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F30" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-26/spity-022-club-dashboard</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="39" customHeight="1">
+      <x:c r="A31" s="2" t="str">
+        <x:v>SPI-27</x:v>
+      </x:c>
+      <x:c r="B31" s="25" t="str">
+        <x:v>SPITY-023: Upload media sécurisé</x:v>
+      </x:c>
+      <x:c r="C31" s="2" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E31" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F31" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-27/spity-023-upload-media-securise</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="39" customHeight="1">
+      <x:c r="A32" s="2" t="str">
+        <x:v>SPI-28</x:v>
+      </x:c>
+      <x:c r="B32" s="25" t="str">
+        <x:v>SPITY-024: Tests unitaires critiques (auth, posts)</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D32" s="2" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E32" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F32" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-28/spity-024-tests-unitaires-critiques-auth-posts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="39" customHeight="1">
+      <x:c r="A33" s="2" t="str">
+        <x:v>SPI-29</x:v>
+      </x:c>
+      <x:c r="B33" s="25" t="str">
+        <x:v>SPITY-025: Sécurité OWASP + accessibilité RGAA</x:v>
+      </x:c>
+      <x:c r="C33" s="2" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D33" s="2" t="str">
+        <x:v>Low</x:v>
+      </x:c>
+      <x:c r="E33" s="2" t="str">
+        <x:v>dorian joly</x:v>
+      </x:c>
+      <x:c r="F33" s="2" t="str">
+        <x:v>https://linear.app/spitywa/issue/SPI-29/spity-025-securite-owasp-accessibilite-rgaa</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="25" customHeight="1">
+      <x:c r="A34" s="2"/>
+      <x:c r="B34" s="2"/>
+      <x:c r="C34" s="2"/>
+      <x:c r="D34" s="2"/>
+      <x:c r="E34" s="2"/>
+      <x:c r="F34" s="2"/>
+    </x:row>
+    <x:row r="35" ht="25" customHeight="1">
+      <x:c r="A35" s="2"/>
+      <x:c r="B35" s="2" t="str">
+        <x:v>Source : https://linear.app/spitywa/team/SPI/all ; transcription datée, détails et limites dans A09.</x:v>
+      </x:c>
+      <x:c r="C35" s="2"/>
+      <x:c r="D35" s="2"/>
+      <x:c r="E35" s="2"/>
+      <x:c r="F35" s="2"/>
+    </x:row>
+    <x:row r="36" ht="25" customHeight="1">
+      <x:c r="A36" s="2"/>
+      <x:c r="B36" s="2" t="str">
+        <x:v>Les données simulées CP / DEV / QA restent distinctes de l’affectation nominale dans Linear.</x:v>
+      </x:c>
+      <x:c r="C36" s="2"/>
+      <x:c r="D36" s="2"/>
+      <x:c r="E36" s="2"/>
+      <x:c r="F36" s="2"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>